<commit_message>
Add more observations to the HICP_EUR
</commit_message>
<xml_diff>
--- a/data/raw/Inflation/HICP_EUR.xlsx
+++ b/data/raw/Inflation/HICP_EUR.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Martina\Documents\Práce\Mezinárodní instituce\OECD_2026_09\embodied-carbon-czech-imports\data\raw\Inflation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7496796-B66F-4A69-AB59-F4982EBFF181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB28B38C-F9B0-4624-B235-8BBBE87FAEF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A3DF72DF-C7A0-40B3-B453-F6BE455B65F6}"/>
   </bookViews>
@@ -426,7 +426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B72D6178-BAB8-47BE-A04B-D11CFB4E7C24}">
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -439,226 +439,269 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>1996</v>
-      </c>
-      <c r="B2">
-        <v>70.260000000000005</v>
-      </c>
+        <v>1990</v>
+      </c>
+      <c r="B2" s="1"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>1997</v>
-      </c>
-      <c r="B3">
-        <v>71.48</v>
-      </c>
+        <v>1991</v>
+      </c>
+      <c r="B3" s="1"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>1998</v>
-      </c>
-      <c r="B4">
-        <v>72.400000000000006</v>
-      </c>
+        <v>1992</v>
+      </c>
+      <c r="B4" s="1"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>1999</v>
-      </c>
-      <c r="B5">
-        <v>73.260000000000005</v>
-      </c>
+        <v>1993</v>
+      </c>
+      <c r="B5" s="1"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>2000</v>
-      </c>
-      <c r="B6">
-        <v>74.650000000000006</v>
-      </c>
+        <v>1994</v>
+      </c>
+      <c r="B6" s="1"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>2001</v>
-      </c>
-      <c r="B7">
-        <v>76.290000000000006</v>
+        <v>1995</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>2002</v>
+        <v>1996</v>
       </c>
       <c r="B8">
-        <v>77.87</v>
+        <v>70.260000000000005</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>2003</v>
+        <v>1997</v>
       </c>
       <c r="B9">
-        <v>79.400000000000006</v>
+        <v>71.48</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>2004</v>
+        <v>1998</v>
       </c>
       <c r="B10">
-        <v>81</v>
+        <v>72.400000000000006</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>2005</v>
+        <v>1999</v>
       </c>
       <c r="B11">
-        <v>82.75</v>
+        <v>73.260000000000005</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>2006</v>
+        <v>2000</v>
       </c>
       <c r="B12">
-        <v>84.58</v>
+        <v>74.650000000000006</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>2007</v>
+        <v>2001</v>
       </c>
       <c r="B13">
-        <v>86.55</v>
+        <v>76.290000000000006</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>2008</v>
+        <v>2002</v>
       </c>
       <c r="B14">
-        <v>89.72</v>
+        <v>77.87</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>2009</v>
+        <v>2003</v>
       </c>
       <c r="B15">
-        <v>90.6</v>
+        <v>79.400000000000006</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>2010</v>
+        <v>2004</v>
       </c>
       <c r="B16">
-        <v>92.49</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>2011</v>
+        <v>2005</v>
       </c>
       <c r="B17">
-        <v>95.36</v>
+        <v>82.75</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>2012</v>
+        <v>2006</v>
       </c>
       <c r="B18">
-        <v>97.88</v>
+        <v>84.58</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>2013</v>
+        <v>2007</v>
       </c>
       <c r="B19">
-        <v>99.35</v>
+        <v>86.55</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>2014</v>
+        <v>2008</v>
       </c>
       <c r="B20">
-        <v>99.9</v>
+        <v>89.72</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>2015</v>
+        <v>2009</v>
       </c>
       <c r="B21">
-        <v>100</v>
+        <v>90.6</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>2016</v>
+        <v>2010</v>
       </c>
       <c r="B22">
-        <v>100.25</v>
+        <v>92.49</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>2017</v>
+        <v>2011</v>
       </c>
       <c r="B23">
-        <v>101.96</v>
+        <v>95.36</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>2018</v>
+        <v>2012</v>
       </c>
       <c r="B24">
-        <v>103.89</v>
+        <v>97.88</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>2019</v>
+        <v>2013</v>
       </c>
       <c r="B25">
-        <v>105.42</v>
+        <v>99.35</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>2020</v>
+        <v>2014</v>
       </c>
       <c r="B26">
-        <v>106.2</v>
+        <v>99.9</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>2021</v>
+        <v>2015</v>
       </c>
       <c r="B27">
-        <v>109.28</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>2022</v>
+        <v>2016</v>
       </c>
       <c r="B28">
-        <v>119.32</v>
+        <v>100.25</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29">
+        <v>2017</v>
+      </c>
+      <c r="B29">
+        <v>101.96</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>2018</v>
+      </c>
+      <c r="B30">
+        <v>103.89</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>2019</v>
+      </c>
+      <c r="B31">
+        <v>105.42</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>2020</v>
+      </c>
+      <c r="B32">
+        <v>106.2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>2021</v>
+      </c>
+      <c r="B33">
+        <v>109.28</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>2022</v>
+      </c>
+      <c r="B34">
+        <v>119.32</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35">
         <v>2023</v>
       </c>
-      <c r="B29">
+      <c r="B35">
         <v>126.91</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>2024</v>
+      </c>
+      <c r="B36">
+        <v>130.21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>